<commit_message>
Six fixes (D-072 am. 9): call GPS on the job page, the house + remote diagnosis in the tech app, Customer_Type__c, job notes fields, call notes rolled onto the job at completion
- callToBoard carries clockLog (live intervals with GPS per tap + geofence); GET /service/jobs/{id}/calls carries the job's geocode.
- Tech job/call views gain remoteDiagnosis + streetViewUrl; GET /service/tech/jobs/{id}/street-view (estimate Lambda, service.tech.read).
- Customer_Type__c: delta field + FLS in service-objects, Solar default in sf-update, Service set/union-added by resolveCustomer, ?type= on the tech customers list.
- Notes_for_Summary__c / Notes_From_Service_Calls__c on the job (generator, package, cache); job-notes.js rolls a Complete call's work/private notes onto them, one block per call, replaced on edit — in the Lambda, never a Flow.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JKYsKWsvaEjKCtvVsKEQnj
</commit_message>
<xml_diff>
--- a/docs/Sundial_Service_Job_Fields_by_Section.xlsx
+++ b/docs/Sundial_Service_Job_Fields_by_Section.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1076,12 +1076,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Office Notes</t>
+          <t>Notes for Summary</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Office_Notes__c</t>
+          <t>Notes_for_Summary__c</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Internal office log - append-only stamped entries (D-065.8). Separate from tech notes per the 9/9 meeting; tech notes live on Service Calls and are shown here read-only. [not cached — detail only]</t>
+          <t>Every Complete call's WORK notes, one block per call (job-notes.js, 2026-09-19) - the raw material for Customer Summary. Lambda-written; the office may edit.</t>
         </is>
       </c>
     </row>
@@ -1103,74 +1103,78 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Customer Summary</t>
+          <t>Notes From Service Calls</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Customer_Summary__c</t>
+          <t>Notes_From_Service_Calls__c</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Long Text(32768)</t>
+          <t>Long Text(131072)</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>The customer-facing paragraph for the receipt and the photo job report. AI-drafted from the calls' Work Notes, office-edited before send. [not cached — detail only]</t>
+          <t>Every Complete call's PRIVATE notes, one block per call (job-notes.js, 2026-09-19). Internal only. Lambda-written; the office may edit.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Context</t>
+          <t>Narrative</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Originating Solar Project</t>
+          <t>Office Notes</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Originating_Solar_Project__c</t>
+          <t>Office_Notes__c</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Lookup(Sundial_Solar__c)</t>
+          <t>Long Text(131072)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Installed system: specs, install date, photos read from here (no Asset object).</t>
+          <t>Internal office log - append-only stamped entries (D-065.8). Separate from tech notes per the 9/9 meeting; tech notes live on Service Calls and are shown here read-only. [not cached — detail only]</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Context</t>
+          <t>Narrative</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Originating Roofing Project</t>
+          <t>Customer Summary</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Originating_Roofing_Project__c</t>
+          <t>Customer_Summary__c</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Lookup(Sundial_Roofing__c)</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr"/>
+          <t>Long Text(32768)</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>The customer-facing paragraph for the receipt and the photo job report. AI-drafted from the calls' Work Notes, office-edited before send. [not cached — detail only]</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1180,76 +1184,72 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Originating Commercial Project</t>
+          <t>Originating Solar Project</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Originating_Commercial_Project__c</t>
+          <t>Originating_Solar_Project__c</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Lookup(Sundial_Commercial__c)</t>
+          <t>Lookup(Sundial_Solar__c)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Phase 3 object - REMOVE from the package if Sundial_Commercial__c is absent.</t>
+          <t>Installed system: specs, install date, photos read from here (no Asset object).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Billing (one payer)</t>
+          <t>Context</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Bill To Type</t>
+          <t>Originating Roofing Project</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Bill_To_Type__c</t>
+          <t>Originating_Roofing_Project__c</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Picklist: Customer / Internal Warranty / Manufacturer / Leasing Partner / Other (default Customer)</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>THE payer for this job (D-072.6). No customer default, no per-visit override. 'Internal Warranty' is the tenant-neutral value for on-us warranty work.</t>
-        </is>
-      </c>
+          <t>Lookup(Sundial_Roofing__c)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Billing (one payer)</t>
+          <t>Context</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Bill To Name</t>
+          <t>Originating Commercial Project</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Bill_To_Name__c</t>
+          <t>Originating_Commercial_Project__c</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Text(255)</t>
+          <t>Lookup(Sundial_Commercial__c)</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Payer name when not the customer (leasing partner, manufacturer). Partner list is tenant config.</t>
+          <t>Phase 3 object - REMOVE from the package if Sundial_Commercial__c is absent.</t>
         </is>
       </c>
     </row>
@@ -1261,130 +1261,130 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
+          <t>Bill To Type</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Bill_To_Type__c</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Picklist: Customer / Internal Warranty / Manufacturer / Leasing Partner / Other (default Customer)</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>THE payer for this job (D-072.6). No customer default, no per-visit override. 'Internal Warranty' is the tenant-neutral value for on-us warranty work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Billing (one payer)</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Bill To Name</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Bill_To_Name__c</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Text(255)</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Payer name when not the customer (leasing partner, manufacturer). Partner list is tenant config.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Billing (one payer)</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
           <t>Billing Reference</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>Billing_Reference__c</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Text(100) · External ID</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>Partner PO / work-order number. External ID (indexed) - 'SunRun calls with THEIR number'; printed on the invoice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>Billing (one payer)</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>Payment Status</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Payment_Status__c</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>Picklist: None / Deposit Paid / Partially Paid / Paid / Refunded (default None)</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>Derived from Service Payments vs invoice total (Lambda/Flow).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>Billing (one payer)</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>Customer Card on File</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>Customer_Card_on_File__c</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>Checkbox (default false)</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>A SetupIntent completed for this customer (mirror of the customer's Stripe state at last check). Cards live in Stripe, never here.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Estimate (read-through)</t>
+          <t>Billing (one payer)</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Estimate Status</t>
+          <t>Payment Status</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Estimate_Status__c</t>
+          <t>Payment_Status__c</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Formula (Text)</t>
+          <t>Picklist: None / Deposit Paid / Partially Paid / Paid / Refunded (default None)</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Cross-object formula - the job list shows it as a column.</t>
+          <t>Derived from Service Payments vs invoice total (Lambda/Flow).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Estimate (read-through)</t>
+          <t>Billing (one payer)</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Estimate Total</t>
+          <t>Customer Card on File</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Estimate_Total__c</t>
+          <t>Customer_Card_on_File__c</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Formula (Currency)</t>
+          <t>Checkbox (default false)</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Cross-object formula onto the living estimate - no sync, no drift (D-072.3).</t>
+          <t>A SetupIntent completed for this customer (mirror of the customer's Stripe state at last check). Cards live in Stripe, never here.</t>
         </is>
       </c>
     </row>
@@ -1396,22 +1396,22 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Estimate Approved Amount</t>
+          <t>Estimate Status</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Estimate_Approved_Amount__c</t>
+          <t>Estimate_Status__c</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Formula (Currency)</t>
+          <t>Formula (Text)</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>What the customer last approved.</t>
+          <t>Cross-object formula - the job list shows it as a column.</t>
         </is>
       </c>
     </row>
@@ -1423,12 +1423,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Estimate Deposit Amount</t>
+          <t>Estimate Total</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Estimate_Deposit_Amount__c</t>
+          <t>Estimate_Total__c</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -1436,61 +1436,61 @@
           <t>Formula (Currency)</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Cross-object formula onto the living estimate - no sync, no drift (D-072.3).</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Time roll-ups</t>
+          <t>Estimate (read-through)</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Total Call Count</t>
+          <t>Estimate Approved Amount</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Total_Call_Count__c</t>
+          <t>Estimate_Approved_Amount__c</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Number(5,0)</t>
+          <t>Formula (Currency)</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Roll-up via record-triggered Flow on Service Call change (D-065.3). Migration writes totals directly.</t>
+          <t>What the customer last approved.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Time roll-ups</t>
+          <t>Estimate (read-through)</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Total Time Minutes</t>
+          <t>Estimate Deposit Amount</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Total_Time_Minutes__c</t>
+          <t>Estimate_Deposit_Amount__c</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Number(9,0)</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>Sum of Service Call durations across all techs (roll-up Flow).</t>
-        </is>
-      </c>
+          <t>Formula (Currency)</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -1500,74 +1500,78 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>First Scheduled Start</t>
+          <t>Total Call Count</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>First_Scheduled_Start__c</t>
+          <t>Total_Call_Count__c</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>Number(5,0)</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Earliest Service Call Scheduled_Start (roll-up Flow) - list sorting.</t>
+          <t>Roll-up via record-triggered Flow on Service Call change (D-065.3). Migration writes totals directly.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Location</t>
+          <t>Time roll-ups</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Geocode Latitude</t>
+          <t>Total Time Minutes</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Geocode_Lat__c</t>
+          <t>Total_Time_Minutes__c</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Number(18,15)</t>
+          <t>Number(9,0)</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Service-address geocode, best-effort at intake; feeds geofence + travel hints.</t>
+          <t>Sum of Service Call durations across all techs (roll-up Flow).</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Location</t>
+          <t>Time roll-ups</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Geocode Longitude</t>
+          <t>First Scheduled Start</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Geocode_Lon__c</t>
+          <t>First_Scheduled_Start__c</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Number(18,15)</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr"/>
+          <t>DateTime</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Earliest Service Call Scheduled_Start (roll-up Flow) - list sorting.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -1577,22 +1581,22 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Geocode Status</t>
+          <t>Geocode Latitude</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Geocode_Status__c</t>
+          <t>Geocode_Lat__c</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Picklist: Pending / Geocoded / Failed / Manual (default Pending)</t>
+          <t>Number(18,15)</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Failed/Manual rows fall back to no geofence rather than blocking clock-ins.</t>
+          <t>Service-address geocode, best-effort at intake; feeds geofence + travel hints.</t>
         </is>
       </c>
     </row>
@@ -1604,20 +1608,70 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
+          <t>Geocode Longitude</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Geocode_Lon__c</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Number(18,15)</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Geocode Status</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Geocode_Status__c</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Picklist: Pending / Geocoded / Failed / Manual (default Pending)</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Failed/Manual rows fall back to no geofence rather than blocking clock-ins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
           <t>Street View Image Key</t>
         </is>
       </c>
-      <c r="C44" s="3" t="inlineStr">
+      <c r="C46" s="3" t="inlineStr">
         <is>
           <t>Street_View_Image_Key__c</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr">
+      <c r="D46" s="3" t="inlineStr">
         <is>
           <t>Text(255)</t>
         </is>
       </c>
-      <c r="E44" s="3" t="inlineStr">
+      <c r="E46" s="3" t="inlineStr">
         <is>
           <t>S3 key of the street-view still fetched once at geocode time (9/9 ask). Blank = none available. [not cached — detail only]</t>
         </is>

</xml_diff>

<commit_message>
Job report + receipt (D-072 am. 10): built section by section on the job, one model / two painters with photos in the PDF, sent + re-sent with a button; /public/reports/{token}; delta package 2026-09-19
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JKYsKWsvaEjKCtvVsKEQnj
</commit_message>
<xml_diff>
--- a/docs/Sundial_Service_Job_Fields_by_Section.xlsx
+++ b/docs/Sundial_Service_Job_Fields_by_Section.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1674,6 +1674,191 @@
       <c r="E46" s="3" t="inlineStr">
         <is>
           <t>S3 key of the street-view still fetched once at geocode time (9/9 ask). Blank = none available. [not cached — detail only]</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Job Report</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Report Sections</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Report_Sections__c</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Long Text(131072)</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>The report as the office built it: JSON { version, sections: [{ id, photoKey, caption }], receipt }. Lambda-written from the portal's Create Report popup; never hand-edited. [not cached — detail only]</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Job Report</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Report Public Token</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Report_Public_Token__c</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Text(128) · External ID</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>The hosted report page's credential (/report/{token}); issued on the first send, renewed on every send. [not cached — detail only]</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Job Report</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Report Token Expires At</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Report_Token_Expires_At__c</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>DateTime</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> [not cached — detail only]</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Job Report</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Report Updated At</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Report_Updated_At__c</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>DateTime</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Last edit of the sections (the job page nudges when it is later than the last send).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Job Report</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Report Sent At</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Report_Sent_At__c</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>DateTime</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Last time the report went to the customer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Job Report</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Report Sent Count</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Report_Sent_Count__c</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Number(18,0)</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Job Report</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Report PDF S3 Key</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Report_PDF_S3_Key__c</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Text(255)</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>SUNDIAL/{jobId}/job-report-{n}.pdf - the PDF of the last send. [not cached — detail only]</t>
         </is>
       </c>
     </row>

</xml_diff>